<commit_message>
alterações novas, lançamento de farmacia
</commit_message>
<xml_diff>
--- a/Base de Dados/ESCRITORIO_PRONTO-teste.xlsx
+++ b/Base de Dados/ESCRITORIO_PRONTO-teste.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\flavi\OneDrive\Desktop\Projeto_RH\Base de Dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F260054D-6C38-4A23-8B10-CDE618EC7FFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21C3164A-796B-4820-A77F-C91C0A0F2DD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -256,9 +256,6 @@
     <t>uchoa</t>
   </si>
   <si>
-    <t>Aparecida Andrea da Silva Castilho</t>
-  </si>
-  <si>
     <t>372.599.748-93</t>
   </si>
   <si>
@@ -664,9 +661,6 @@
     <t>460.458.258-02</t>
   </si>
   <si>
-    <t xml:space="preserve">Mara Ivanirlly Dos Santos Miranda </t>
-  </si>
-  <si>
     <t>091.035.273-95</t>
   </si>
   <si>
@@ -965,6 +959,12 @@
   </si>
   <si>
     <t>Carlos Henrique Gimenes Martins</t>
+  </si>
+  <si>
+    <t>Aparecida Andrea Castilho</t>
+  </si>
+  <si>
+    <t>Mara Ivanirlly Santos</t>
   </si>
 </sst>
 </file>
@@ -976,7 +976,7 @@
     <numFmt numFmtId="165" formatCode="[h]:mm"/>
     <numFmt numFmtId="166" formatCode="0.000%"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1040,6 +1040,13 @@
     </font>
     <font>
       <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1234,7 +1241,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="88">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1423,6 +1430,7 @@
     <xf numFmtId="165" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="20" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="5" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2207,7 +2215,7 @@
         <v>1279</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="C10" s="76">
         <v>38925</v>
@@ -2494,13 +2502,13 @@
         <v>1280</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>57</v>
+        <v>292</v>
       </c>
       <c r="C14" s="76">
         <v>32302</v>
       </c>
       <c r="D14" s="77" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E14" s="78"/>
       <c r="F14" s="79">
@@ -2565,13 +2573,13 @@
         <v>1227</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C15" s="76">
         <v>37089</v>
       </c>
       <c r="D15" s="77" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E15" s="78"/>
       <c r="F15" s="79">
@@ -2636,13 +2644,13 @@
         <v>1165</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C16" s="76">
         <v>34139</v>
       </c>
       <c r="D16" s="77" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E16" s="78"/>
       <c r="F16" s="79">
@@ -2707,13 +2715,13 @@
         <v>1293</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C17" s="76">
         <v>36794</v>
       </c>
       <c r="D17" s="77" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E17" s="78"/>
       <c r="F17" s="79">
@@ -2731,7 +2739,7 @@
         <v>38</v>
       </c>
       <c r="J17" s="55" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="K17" s="56">
         <v>2158</v>
@@ -2778,13 +2786,13 @@
         <v>1075</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C18" s="76">
         <v>29315</v>
       </c>
       <c r="D18" s="77" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E18" s="78">
         <v>44866</v>
@@ -2801,10 +2809,10 @@
         <v>45780</v>
       </c>
       <c r="I18" s="55" t="s">
+        <v>67</v>
+      </c>
+      <c r="J18" s="55" t="s">
         <v>68</v>
-      </c>
-      <c r="J18" s="55" t="s">
-        <v>69</v>
       </c>
       <c r="K18" s="56">
         <v>2158</v>
@@ -2851,13 +2859,13 @@
         <v>1040</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C19" s="76">
         <v>30929</v>
       </c>
       <c r="D19" s="77" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E19" s="78">
         <v>44838</v>
@@ -2874,7 +2882,7 @@
         <v>45543</v>
       </c>
       <c r="I19" s="55" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J19" s="55" t="s">
         <v>42</v>
@@ -2926,13 +2934,13 @@
         <v>1134</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="C20" s="76">
         <v>37383</v>
       </c>
       <c r="D20" s="77" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E20" s="78"/>
       <c r="F20" s="79">
@@ -2950,7 +2958,7 @@
         <v>38</v>
       </c>
       <c r="J20" s="55" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="K20" s="56">
         <v>2158</v>
@@ -2997,13 +3005,13 @@
         <v>1215</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C21" s="76">
         <v>34064</v>
       </c>
       <c r="D21" s="77" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E21" s="78"/>
       <c r="F21" s="79">
@@ -3068,13 +3076,13 @@
         <v>1254</v>
       </c>
       <c r="B22" s="15" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C22" s="76">
         <v>38378</v>
       </c>
       <c r="D22" s="77" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E22" s="78"/>
       <c r="F22" s="79">
@@ -3092,7 +3100,7 @@
         <v>38</v>
       </c>
       <c r="J22" s="55" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="K22" s="56">
         <v>2158</v>
@@ -3139,13 +3147,13 @@
         <v>1257</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C23" s="76">
         <v>33488</v>
       </c>
       <c r="D23" s="77" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E23" s="78"/>
       <c r="F23" s="79">
@@ -3210,13 +3218,13 @@
         <v>1062</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C24" s="76">
         <v>32573</v>
       </c>
       <c r="D24" s="77" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E24" s="78">
         <v>45483</v>
@@ -3285,13 +3293,13 @@
         <v>1269</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C25" s="76">
         <v>32505</v>
       </c>
       <c r="D25" s="77" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E25" s="78"/>
       <c r="F25" s="79">
@@ -3309,7 +3317,7 @@
         <v>38</v>
       </c>
       <c r="J25" s="55" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="K25" s="56">
         <v>2158</v>
@@ -3356,13 +3364,13 @@
         <v>1282</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C26" s="76">
         <v>34034</v>
       </c>
       <c r="D26" s="77" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E26" s="78"/>
       <c r="F26" s="79">
@@ -3427,13 +3435,13 @@
         <v>1262</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C27" s="76">
         <v>38114</v>
       </c>
       <c r="D27" s="77" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E27" s="78"/>
       <c r="F27" s="79">
@@ -3498,13 +3506,13 @@
         <v>1297</v>
       </c>
       <c r="B28" s="15" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C28" s="76">
         <v>35286</v>
       </c>
       <c r="D28" s="77" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E28" s="78"/>
       <c r="F28" s="79">
@@ -3522,7 +3530,7 @@
         <v>38</v>
       </c>
       <c r="J28" s="55" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="K28" s="56">
         <v>2158</v>
@@ -3569,13 +3577,13 @@
         <v>1006</v>
       </c>
       <c r="B29" s="15" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C29" s="76">
         <v>34083</v>
       </c>
       <c r="D29" s="77" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E29" s="78">
         <v>44927</v>
@@ -3592,7 +3600,7 @@
         <v>45167</v>
       </c>
       <c r="I29" s="55" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="J29" s="55" t="s">
         <v>53</v>
@@ -3644,13 +3652,13 @@
         <v>1290</v>
       </c>
       <c r="B30" s="15" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C30" s="76">
         <v>38300</v>
       </c>
       <c r="D30" s="77" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E30" s="78"/>
       <c r="F30" s="79">
@@ -3706,13 +3714,13 @@
         <v>1080</v>
       </c>
       <c r="B31" s="15" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C31" s="76">
         <v>33127</v>
       </c>
       <c r="D31" s="77" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E31" s="78">
         <v>45684</v>
@@ -3729,10 +3737,10 @@
         <v>45808</v>
       </c>
       <c r="I31" s="55" t="s">
+        <v>97</v>
+      </c>
+      <c r="J31" s="55" t="s">
         <v>98</v>
-      </c>
-      <c r="J31" s="55" t="s">
-        <v>99</v>
       </c>
       <c r="K31" s="56">
         <v>3045.9</v>
@@ -3779,13 +3787,13 @@
         <v>1018</v>
       </c>
       <c r="B32" s="15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C32" s="76">
         <v>27693</v>
       </c>
       <c r="D32" s="77" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E32" s="78">
         <v>45170</v>
@@ -3802,10 +3810,10 @@
         <v>45297</v>
       </c>
       <c r="I32" s="55" t="s">
+        <v>67</v>
+      </c>
+      <c r="J32" s="55" t="s">
         <v>68</v>
-      </c>
-      <c r="J32" s="55" t="s">
-        <v>69</v>
       </c>
       <c r="K32" s="56">
         <v>2158</v>
@@ -3852,13 +3860,13 @@
         <v>1296</v>
       </c>
       <c r="B33" s="15" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C33" s="76">
         <v>30043</v>
       </c>
       <c r="D33" s="77" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E33" s="78"/>
       <c r="F33" s="79">
@@ -3876,7 +3884,7 @@
         <v>38</v>
       </c>
       <c r="J33" s="55" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="K33" s="56">
         <v>2158</v>
@@ -3923,13 +3931,13 @@
         <v>1265</v>
       </c>
       <c r="B34" s="15" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C34" s="76">
         <v>35501</v>
       </c>
       <c r="D34" s="77" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E34" s="78"/>
       <c r="F34" s="79">
@@ -3947,7 +3955,7 @@
         <v>38</v>
       </c>
       <c r="J34" s="55" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="K34" s="56">
         <v>2158</v>
@@ -3994,13 +4002,13 @@
         <v>1283</v>
       </c>
       <c r="B35" s="15" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C35" s="76">
         <v>37025</v>
       </c>
       <c r="D35" s="77" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E35" s="78"/>
       <c r="F35" s="79">
@@ -4065,7 +4073,7 @@
         <v>1271</v>
       </c>
       <c r="B36" s="15" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C36" s="76">
         <v>35750</v>
@@ -4089,7 +4097,7 @@
         <v>38</v>
       </c>
       <c r="J36" s="55" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="K36" s="56">
         <v>2158</v>
@@ -4136,13 +4144,13 @@
         <v>1097</v>
       </c>
       <c r="B37" s="15" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C37" s="76">
         <v>32921</v>
       </c>
       <c r="D37" s="77" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E37" s="78"/>
       <c r="F37" s="79">
@@ -4157,7 +4165,7 @@
         <v>45837</v>
       </c>
       <c r="I37" s="55" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J37" s="55" t="s">
         <v>39</v>
@@ -4207,13 +4215,13 @@
         <v>1224</v>
       </c>
       <c r="B38" s="15" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C38" s="76">
         <v>29930</v>
       </c>
       <c r="D38" s="77" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E38" s="78"/>
       <c r="F38" s="79">
@@ -4231,7 +4239,7 @@
         <v>38</v>
       </c>
       <c r="J38" s="55" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="K38" s="56">
         <v>2158</v>
@@ -4278,13 +4286,13 @@
         <v>1299</v>
       </c>
       <c r="B39" s="15" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C39" s="76">
         <v>36485</v>
       </c>
       <c r="D39" s="77" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E39" s="78"/>
       <c r="F39" s="79">
@@ -4302,7 +4310,7 @@
         <v>38</v>
       </c>
       <c r="J39" s="55" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="K39" s="56">
         <v>2158</v>
@@ -4349,13 +4357,13 @@
         <v>1195</v>
       </c>
       <c r="B40" s="15" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C40" s="76">
         <v>37361</v>
       </c>
       <c r="D40" s="77" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E40" s="78"/>
       <c r="F40" s="79">
@@ -4420,13 +4428,13 @@
         <v>1233</v>
       </c>
       <c r="B41" s="15" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C41" s="76">
         <v>33088</v>
       </c>
       <c r="D41" s="77" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E41" s="78"/>
       <c r="F41" s="79">
@@ -4491,13 +4499,13 @@
         <v>1277</v>
       </c>
       <c r="B42" s="15" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C42" s="76">
         <v>34866</v>
       </c>
       <c r="D42" s="77" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E42" s="78"/>
       <c r="F42" s="79">
@@ -4562,13 +4570,13 @@
         <v>1216</v>
       </c>
       <c r="B43" s="30" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C43" s="76">
         <v>36697</v>
       </c>
       <c r="D43" s="77" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E43" s="78"/>
       <c r="F43" s="79">
@@ -4583,7 +4591,7 @@
         <v>46134</v>
       </c>
       <c r="I43" s="55" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="J43" s="55" t="s">
         <v>45</v>
@@ -4633,13 +4641,13 @@
         <v>1082</v>
       </c>
       <c r="B44" s="15" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C44" s="76">
         <v>32398</v>
       </c>
       <c r="D44" s="77" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E44" s="78"/>
       <c r="F44" s="79">
@@ -4704,13 +4712,13 @@
         <v>1121</v>
       </c>
       <c r="B45" s="15" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C45" s="76">
         <v>38663</v>
       </c>
       <c r="D45" s="77" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E45" s="78"/>
       <c r="F45" s="79">
@@ -4775,13 +4783,13 @@
         <v>1019</v>
       </c>
       <c r="B46" s="15" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C46" s="76">
         <v>36927</v>
       </c>
       <c r="D46" s="77" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E46" s="78">
         <v>44812</v>
@@ -4798,10 +4806,10 @@
         <v>45297</v>
       </c>
       <c r="I46" s="55" t="s">
+        <v>132</v>
+      </c>
+      <c r="J46" s="55" t="s">
         <v>133</v>
-      </c>
-      <c r="J46" s="55" t="s">
-        <v>134</v>
       </c>
       <c r="K46" s="56">
         <v>3195.3</v>
@@ -4850,13 +4858,13 @@
         <v>1104</v>
       </c>
       <c r="B47" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C47" s="76">
         <v>38176</v>
       </c>
       <c r="D47" s="77" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E47" s="78">
         <v>45756</v>
@@ -4873,10 +4881,10 @@
         <v>45850</v>
       </c>
       <c r="I47" s="55" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="J47" s="55" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="K47" s="56">
         <v>2158</v>
@@ -4923,13 +4931,13 @@
         <v>1194</v>
       </c>
       <c r="B48" s="15" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C48" s="76">
         <v>37265</v>
       </c>
       <c r="D48" s="77" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E48" s="78"/>
       <c r="F48" s="79">
@@ -4994,13 +5002,13 @@
         <v>1181</v>
       </c>
       <c r="B49" s="15" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C49" s="76">
         <v>36141</v>
       </c>
       <c r="D49" s="77" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E49" s="78"/>
       <c r="F49" s="79">
@@ -5018,7 +5026,7 @@
         <v>38</v>
       </c>
       <c r="J49" s="55" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="K49" s="56">
         <v>2158</v>
@@ -5065,13 +5073,13 @@
         <v>1135</v>
       </c>
       <c r="B50" s="15" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C50" s="76">
         <v>23787</v>
       </c>
       <c r="D50" s="77" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E50" s="78">
         <v>44044</v>
@@ -5140,13 +5148,13 @@
         <v>1172</v>
       </c>
       <c r="B51" s="15" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C51" s="76">
         <v>33969</v>
       </c>
       <c r="D51" s="77" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E51" s="78"/>
       <c r="F51" s="79">
@@ -5211,13 +5219,13 @@
         <v>1284</v>
       </c>
       <c r="B52" s="15" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C52" s="76">
         <v>39442</v>
       </c>
       <c r="D52" s="77" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E52" s="78"/>
       <c r="F52" s="79">
@@ -5282,13 +5290,13 @@
         <v>1218</v>
       </c>
       <c r="B53" s="15" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C53" s="76">
         <v>30394</v>
       </c>
       <c r="D53" s="77" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E53" s="78"/>
       <c r="F53" s="79">
@@ -5353,13 +5361,13 @@
         <v>1060</v>
       </c>
       <c r="B54" s="15" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C54" s="76">
         <v>35833</v>
       </c>
       <c r="D54" s="77" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E54" s="78">
         <v>45495</v>
@@ -5428,13 +5436,13 @@
         <v>1273</v>
       </c>
       <c r="B55" s="15" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C55" s="76">
         <v>37631</v>
       </c>
       <c r="D55" s="77" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E55" s="78"/>
       <c r="F55" s="79">
@@ -5452,7 +5460,7 @@
         <v>38</v>
       </c>
       <c r="J55" s="55" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="K55" s="56">
         <v>2158</v>
@@ -5499,13 +5507,13 @@
         <v>1090</v>
       </c>
       <c r="B56" s="15" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C56" s="76">
         <v>36611</v>
       </c>
       <c r="D56" s="77" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E56" s="78">
         <v>45733</v>
@@ -5572,13 +5580,13 @@
         <v>1223</v>
       </c>
       <c r="B57" s="15" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C57" s="76">
         <v>32548</v>
       </c>
       <c r="D57" s="77" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E57" s="78"/>
       <c r="F57" s="79">
@@ -5593,10 +5601,10 @@
         <v>46141</v>
       </c>
       <c r="I57" s="55" t="s">
+        <v>156</v>
+      </c>
+      <c r="J57" s="55" t="s">
         <v>157</v>
-      </c>
-      <c r="J57" s="55" t="s">
-        <v>158</v>
       </c>
       <c r="K57" s="56">
         <v>2250</v>
@@ -5643,13 +5651,13 @@
         <v>1253</v>
       </c>
       <c r="B58" s="15" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C58" s="76">
         <v>39248</v>
       </c>
       <c r="D58" s="77" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="E58" s="78"/>
       <c r="F58" s="79">
@@ -5667,7 +5675,7 @@
         <v>38</v>
       </c>
       <c r="J58" s="55" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="K58" s="56">
         <v>2158</v>
@@ -5714,13 +5722,13 @@
         <v>1213</v>
       </c>
       <c r="B59" s="15" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C59" s="76">
         <v>35665</v>
       </c>
       <c r="D59" s="77" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E59" s="78"/>
       <c r="F59" s="79">
@@ -5738,7 +5746,7 @@
         <v>38</v>
       </c>
       <c r="J59" s="59" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="K59" s="60">
         <v>2158</v>
@@ -5785,13 +5793,13 @@
         <v>1274</v>
       </c>
       <c r="B60" s="15" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C60" s="76">
         <v>37868</v>
       </c>
       <c r="D60" s="77" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E60" s="78"/>
       <c r="F60" s="79">
@@ -5856,13 +5864,13 @@
         <v>1285</v>
       </c>
       <c r="B61" s="15" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C61" s="76">
         <v>30273</v>
       </c>
       <c r="D61" s="77" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E61" s="78"/>
       <c r="F61" s="79">
@@ -5927,13 +5935,13 @@
         <v>1222</v>
       </c>
       <c r="B62" s="15" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C62" s="76">
         <v>30857</v>
       </c>
       <c r="D62" s="77" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E62" s="78"/>
       <c r="F62" s="79">
@@ -5998,13 +6006,13 @@
         <v>1149</v>
       </c>
       <c r="B63" s="15" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C63" s="76">
         <v>28244</v>
       </c>
       <c r="D63" s="77" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E63" s="78">
         <v>44652</v>
@@ -6073,13 +6081,13 @@
         <v>1303</v>
       </c>
       <c r="B64" s="15" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C64" s="76">
         <v>37371</v>
       </c>
       <c r="D64" s="77" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E64" s="78"/>
       <c r="F64" s="79">
@@ -6097,7 +6105,7 @@
         <v>38</v>
       </c>
       <c r="J64" s="55" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="K64" s="56">
         <v>3195.3</v>
@@ -6141,13 +6149,13 @@
         <v>1152</v>
       </c>
       <c r="B65" s="15" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C65" s="76">
         <v>35717</v>
       </c>
       <c r="D65" s="77" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="E65" s="78"/>
       <c r="F65" s="79">
@@ -6212,13 +6220,13 @@
         <v>1231</v>
       </c>
       <c r="B66" s="15" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C66" s="76">
         <v>35679</v>
       </c>
       <c r="D66" s="77" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E66" s="78"/>
       <c r="F66" s="79">
@@ -6236,7 +6244,7 @@
         <v>38</v>
       </c>
       <c r="J66" s="55" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="K66" s="56">
         <v>2158</v>
@@ -6283,13 +6291,13 @@
         <v>1092</v>
       </c>
       <c r="B67" s="15" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C67" s="76">
         <v>37999</v>
       </c>
       <c r="D67" s="77" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E67" s="78">
         <v>45733</v>
@@ -6306,7 +6314,7 @@
         <v>45837</v>
       </c>
       <c r="I67" s="55" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J67" s="55" t="s">
         <v>39</v>
@@ -6356,13 +6364,13 @@
         <v>1286</v>
       </c>
       <c r="B68" s="15" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C68" s="76">
         <v>36009</v>
       </c>
       <c r="D68" s="77" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="E68" s="78"/>
       <c r="F68" s="79">
@@ -6427,13 +6435,13 @@
         <v>1132</v>
       </c>
       <c r="B69" s="15" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C69" s="76">
         <v>34958</v>
       </c>
       <c r="D69" s="77" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E69" s="78">
         <v>45684</v>
@@ -6450,10 +6458,10 @@
         <v>45899</v>
       </c>
       <c r="I69" s="55" t="s">
+        <v>182</v>
+      </c>
+      <c r="J69" s="55" t="s">
         <v>183</v>
-      </c>
-      <c r="J69" s="55" t="s">
-        <v>184</v>
       </c>
       <c r="K69" s="56">
         <v>3195</v>
@@ -6500,13 +6508,13 @@
         <v>1300</v>
       </c>
       <c r="B70" s="15" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C70" s="76">
         <v>38937</v>
       </c>
       <c r="D70" s="77" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E70" s="78"/>
       <c r="F70" s="79">
@@ -6524,7 +6532,7 @@
         <v>38</v>
       </c>
       <c r="J70" s="55" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="K70" s="56">
         <v>2158</v>
@@ -6571,13 +6579,13 @@
         <v>1251</v>
       </c>
       <c r="B71" s="15" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C71" s="76">
         <v>39302</v>
       </c>
       <c r="D71" s="77" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="E71" s="78"/>
       <c r="F71" s="79">
@@ -6595,7 +6603,7 @@
         <v>38</v>
       </c>
       <c r="J71" s="55" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="K71" s="56">
         <v>2158</v>
@@ -6642,13 +6650,13 @@
         <v>1258</v>
       </c>
       <c r="B72" s="15" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C72" s="76">
         <v>37132</v>
       </c>
       <c r="D72" s="77" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="E72" s="78"/>
       <c r="F72" s="79">
@@ -6713,13 +6721,13 @@
         <v>1276</v>
       </c>
       <c r="B73" s="15" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C73" s="76">
         <v>35995</v>
       </c>
       <c r="D73" s="77" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E73" s="78"/>
       <c r="F73" s="79">
@@ -6784,13 +6792,13 @@
         <v>1246</v>
       </c>
       <c r="B74" s="15" t="s">
-        <v>193</v>
+        <v>293</v>
       </c>
       <c r="C74" s="76">
         <v>38227</v>
       </c>
       <c r="D74" s="77" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E74" s="78"/>
       <c r="F74" s="79">
@@ -6855,13 +6863,13 @@
         <v>1207</v>
       </c>
       <c r="B75" s="15" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C75" s="76">
         <v>34094</v>
       </c>
       <c r="D75" s="77" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="E75" s="78"/>
       <c r="F75" s="79">
@@ -6879,7 +6887,7 @@
         <v>38</v>
       </c>
       <c r="J75" s="55" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="K75" s="56">
         <v>2158</v>
@@ -6926,13 +6934,13 @@
         <v>1203</v>
       </c>
       <c r="B76" s="15" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C76" s="76">
         <v>37153</v>
       </c>
       <c r="D76" s="77" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="E76" s="78"/>
       <c r="F76" s="79">
@@ -6950,7 +6958,7 @@
         <v>38</v>
       </c>
       <c r="J76" s="55" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="K76" s="56">
         <v>2158</v>
@@ -6997,13 +7005,13 @@
         <v>1155</v>
       </c>
       <c r="B77" s="15" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="C77" s="76">
         <v>29892</v>
       </c>
       <c r="D77" s="77" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="E77" s="78"/>
       <c r="F77" s="79">
@@ -7068,13 +7076,13 @@
         <v>1015</v>
       </c>
       <c r="B78" s="15" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C78" s="76">
         <v>36728</v>
       </c>
       <c r="D78" s="77" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="E78" s="78">
         <v>44805</v>
@@ -7091,10 +7099,10 @@
         <v>45251</v>
       </c>
       <c r="I78" s="55" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="J78" s="55" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="K78" s="56">
         <v>2373.8000000000002</v>
@@ -7142,14 +7150,14 @@
       <c r="A79" s="14">
         <v>1235</v>
       </c>
-      <c r="B79" s="15" t="s">
-        <v>203</v>
+      <c r="B79" s="88" t="s">
+        <v>201</v>
       </c>
       <c r="C79" s="76">
         <v>38217</v>
       </c>
       <c r="D79" s="77" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="E79" s="78"/>
       <c r="F79" s="79">
@@ -7214,13 +7222,13 @@
         <v>1267</v>
       </c>
       <c r="B80" s="15" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C80" s="76">
         <v>30690</v>
       </c>
       <c r="D80" s="77" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="E80" s="78"/>
       <c r="F80" s="79">
@@ -7285,13 +7293,13 @@
         <v>1130</v>
       </c>
       <c r="B81" s="15" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="C81" s="76">
         <v>32401</v>
       </c>
       <c r="D81" s="77" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="E81" s="78">
         <v>44316</v>
@@ -7308,7 +7316,7 @@
         <v>45903</v>
       </c>
       <c r="I81" s="55" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="J81" s="55" t="s">
         <v>45</v>
@@ -7360,13 +7368,13 @@
         <v>1238</v>
       </c>
       <c r="B82" s="15" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="C82" s="76">
         <v>33766</v>
       </c>
       <c r="D82" s="77" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="E82" s="78"/>
       <c r="F82" s="79">
@@ -7384,7 +7392,7 @@
         <v>38</v>
       </c>
       <c r="J82" s="55" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="K82" s="56">
         <v>2158</v>
@@ -7431,13 +7439,13 @@
         <v>1153</v>
       </c>
       <c r="B83" s="15" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="C83" s="76">
         <v>32151</v>
       </c>
       <c r="D83" s="77" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="E83" s="78">
         <v>44228</v>
@@ -7506,13 +7514,13 @@
         <v>1302</v>
       </c>
       <c r="B84" s="15" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="C84" s="76">
         <v>30568</v>
       </c>
       <c r="D84" s="77" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="E84" s="78"/>
       <c r="F84" s="79">
@@ -7574,13 +7582,13 @@
         <v>1201</v>
       </c>
       <c r="B85" s="15" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="C85" s="76">
         <v>34187</v>
       </c>
       <c r="D85" s="77" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="E85" s="78"/>
       <c r="F85" s="79">
@@ -7598,7 +7606,7 @@
         <v>38</v>
       </c>
       <c r="J85" s="55" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="K85" s="56">
         <v>2158</v>
@@ -7645,13 +7653,13 @@
         <v>1022</v>
       </c>
       <c r="B86" s="15" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="C86" s="76">
         <v>26896</v>
       </c>
       <c r="D86" s="77" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="E86" s="78">
         <v>44774</v>
@@ -7720,13 +7728,13 @@
         <v>1239</v>
       </c>
       <c r="B87" s="15" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="C87" s="76">
         <v>31709</v>
       </c>
       <c r="D87" s="77" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="E87" s="78"/>
       <c r="F87" s="79">
@@ -7744,7 +7752,7 @@
         <v>38</v>
       </c>
       <c r="J87" s="55" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="K87" s="56">
         <v>2158</v>
@@ -7791,13 +7799,13 @@
         <v>1042</v>
       </c>
       <c r="B88" s="15" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="C88" s="76">
         <v>29583</v>
       </c>
       <c r="D88" s="77" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="E88" s="78">
         <v>45411</v>
@@ -7866,13 +7874,13 @@
         <v>1275</v>
       </c>
       <c r="B89" s="15" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="C89" s="76">
         <v>36349</v>
       </c>
       <c r="D89" s="77" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="E89" s="78"/>
       <c r="F89" s="79">
@@ -7890,7 +7898,7 @@
         <v>38</v>
       </c>
       <c r="J89" s="55" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="K89" s="56">
         <v>2158</v>
@@ -7937,13 +7945,13 @@
         <v>1237</v>
       </c>
       <c r="B90" s="15" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="C90" s="76">
         <v>33175</v>
       </c>
       <c r="D90" s="77" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="E90" s="78"/>
       <c r="F90" s="79">
@@ -8008,13 +8016,13 @@
         <v>1266</v>
       </c>
       <c r="B91" s="15" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C91" s="76">
         <v>38151</v>
       </c>
       <c r="D91" s="77" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="E91" s="78"/>
       <c r="F91" s="79">
@@ -8079,13 +8087,13 @@
         <v>1295</v>
       </c>
       <c r="B92" s="15" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="C92" s="76">
         <v>39579</v>
       </c>
       <c r="D92" s="77" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="E92" s="78"/>
       <c r="F92" s="79">
@@ -8103,7 +8111,7 @@
         <v>38</v>
       </c>
       <c r="J92" s="55" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="K92" s="56">
         <v>2158</v>
@@ -8147,13 +8155,13 @@
         <v>1168</v>
       </c>
       <c r="B93" s="15" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="C93" s="76">
         <v>37321</v>
       </c>
       <c r="D93" s="77" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="E93" s="78"/>
       <c r="F93" s="79">
@@ -8218,13 +8226,13 @@
         <v>1123</v>
       </c>
       <c r="B94" s="15" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C94" s="76">
         <v>33822</v>
       </c>
       <c r="D94" s="77" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="E94" s="78"/>
       <c r="F94" s="79">
@@ -8289,13 +8297,13 @@
         <v>1117</v>
       </c>
       <c r="B95" s="15" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="C95" s="76">
         <v>38871</v>
       </c>
       <c r="D95" s="77" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="E95" s="78"/>
       <c r="F95" s="79">
@@ -8310,7 +8318,7 @@
         <v>45868</v>
       </c>
       <c r="I95" s="55" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="J95" s="55" t="s">
         <v>39</v>
@@ -8360,13 +8368,13 @@
         <v>1179</v>
       </c>
       <c r="B96" s="15" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C96" s="76">
         <v>36156</v>
       </c>
       <c r="D96" s="77" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="E96" s="78"/>
       <c r="F96" s="79">
@@ -8431,13 +8439,13 @@
         <v>1147</v>
       </c>
       <c r="B97" s="15" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C97" s="76">
         <v>27039</v>
       </c>
       <c r="D97" s="77" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="E97" s="78"/>
       <c r="F97" s="79">
@@ -8502,13 +8510,13 @@
         <v>1041</v>
       </c>
       <c r="B98" s="15" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="C98" s="76">
         <v>32265</v>
       </c>
       <c r="D98" s="77" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="E98" s="78">
         <v>45412</v>
@@ -8528,7 +8536,7 @@
         <v>33</v>
       </c>
       <c r="J98" s="55" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="K98" s="56">
         <v>3195.3</v>
@@ -8577,13 +8585,13 @@
         <v>1048</v>
       </c>
       <c r="B99" s="15" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="C99" s="76">
         <v>32275</v>
       </c>
       <c r="D99" s="77" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="E99" s="78">
         <v>45420</v>
@@ -8652,13 +8660,13 @@
         <v>1118</v>
       </c>
       <c r="B100" s="15" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="C100" s="76">
         <v>34310</v>
       </c>
       <c r="D100" s="77" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="E100" s="78">
         <v>45748</v>
@@ -8675,10 +8683,10 @@
         <v>45868</v>
       </c>
       <c r="I100" s="55" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="J100" s="55" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="K100" s="56">
         <v>6390.6</v>
@@ -8727,13 +8735,13 @@
         <v>1225</v>
       </c>
       <c r="B101" s="15" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="C101" s="76">
         <v>36920</v>
       </c>
       <c r="D101" s="77" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="E101" s="78"/>
       <c r="F101" s="79">
@@ -8748,10 +8756,10 @@
         <v>46145</v>
       </c>
       <c r="I101" s="55" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="J101" s="55" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="K101" s="56">
         <v>2158</v>
@@ -8798,13 +8806,13 @@
         <v>1230</v>
       </c>
       <c r="B102" s="15" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="C102" s="76">
         <v>26462</v>
       </c>
       <c r="D102" s="77" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="E102" s="78"/>
       <c r="F102" s="79">
@@ -8869,13 +8877,13 @@
         <v>1004</v>
       </c>
       <c r="B103" s="15" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C103" s="76">
         <v>29019</v>
       </c>
       <c r="D103" s="77" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="E103" s="78">
         <v>45017</v>
@@ -8892,10 +8900,10 @@
         <v>45167</v>
       </c>
       <c r="I103" s="55" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="J103" s="55" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="K103" s="56">
         <v>5006</v>
@@ -8944,13 +8952,13 @@
         <v>1232</v>
       </c>
       <c r="B104" s="15" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="C104" s="76">
         <v>39483</v>
       </c>
       <c r="D104" s="77" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="E104" s="78"/>
       <c r="F104" s="79">
@@ -9015,13 +9023,13 @@
         <v>1093</v>
       </c>
       <c r="B105" s="15" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="C105" s="76">
         <v>38161</v>
       </c>
       <c r="D105" s="77" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="E105" s="78"/>
       <c r="F105" s="79">
@@ -9086,13 +9094,13 @@
         <v>1288</v>
       </c>
       <c r="B106" s="15" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="C106" s="76">
         <v>31476</v>
       </c>
       <c r="D106" s="77" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="E106" s="78"/>
       <c r="F106" s="79">
@@ -9157,13 +9165,13 @@
         <v>1289</v>
       </c>
       <c r="B107" s="15" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C107" s="76">
         <v>36426</v>
       </c>
       <c r="D107" s="77" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="E107" s="78"/>
       <c r="F107" s="79">
@@ -9228,13 +9236,13 @@
         <v>1270</v>
       </c>
       <c r="B108" s="15" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="C108" s="76">
         <v>36939</v>
       </c>
       <c r="D108" s="77" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="E108" s="78"/>
       <c r="F108" s="79">
@@ -9252,7 +9260,7 @@
         <v>38</v>
       </c>
       <c r="J108" s="55" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="K108" s="56">
         <v>2158</v>
@@ -9299,13 +9307,13 @@
         <v>1214</v>
       </c>
       <c r="B109" s="15" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="C109" s="76">
         <v>33917</v>
       </c>
       <c r="D109" s="77" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="E109" s="78"/>
       <c r="F109" s="79">
@@ -9323,7 +9331,7 @@
         <v>38</v>
       </c>
       <c r="J109" s="55" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="K109" s="56">
         <v>2158</v>
@@ -9370,13 +9378,13 @@
         <v>1136</v>
       </c>
       <c r="B110" s="15" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C110" s="76">
         <v>39498</v>
       </c>
       <c r="D110" s="77" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="E110" s="78"/>
       <c r="F110" s="79">
@@ -9441,13 +9449,13 @@
         <v>1241</v>
       </c>
       <c r="B111" s="15" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="C111" s="76">
         <v>30409</v>
       </c>
       <c r="D111" s="77" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="E111" s="78"/>
       <c r="F111" s="79">
@@ -9512,13 +9520,13 @@
         <v>1301</v>
       </c>
       <c r="B112" s="15" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="C112" s="76">
         <v>38377</v>
       </c>
       <c r="D112" s="77" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="E112" s="78"/>
       <c r="F112" s="79">
@@ -9583,13 +9591,13 @@
         <v>1226</v>
       </c>
       <c r="B113" s="15" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C113" s="76">
         <v>35419</v>
       </c>
       <c r="D113" s="77" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="E113" s="78"/>
       <c r="F113" s="79">
@@ -9607,7 +9615,7 @@
         <v>38</v>
       </c>
       <c r="J113" s="55" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="K113" s="56">
         <v>2158</v>
@@ -9654,13 +9662,13 @@
         <v>1291</v>
       </c>
       <c r="B114" s="15" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="C114" s="76">
         <v>36514</v>
       </c>
       <c r="D114" s="77" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="E114" s="78"/>
       <c r="F114" s="79">
@@ -9678,7 +9686,7 @@
         <v>38</v>
       </c>
       <c r="J114" s="55" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="K114" s="56">
         <v>2158</v>
@@ -9725,13 +9733,13 @@
         <v>1003</v>
       </c>
       <c r="B115" s="15" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C115" s="76">
         <v>32989</v>
       </c>
       <c r="D115" s="77" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="E115" s="78">
         <v>44927</v>
@@ -9748,7 +9756,7 @@
         <v>45167</v>
       </c>
       <c r="I115" s="55" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="J115" s="55" t="s">
         <v>45</v>
@@ -9800,7 +9808,7 @@
         <v>1245</v>
       </c>
       <c r="B116" s="41" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="C116" s="76" t="e">
         <v>#N/A</v>
@@ -9824,7 +9832,7 @@
         <v>#N/A</v>
       </c>
       <c r="J116" s="61" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="K116" s="62">
         <v>2158</v>
@@ -9871,13 +9879,13 @@
         <v>1263</v>
       </c>
       <c r="B117" s="30" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="C117" s="76">
         <v>38990</v>
       </c>
       <c r="D117" s="77" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="E117" s="78"/>
       <c r="F117" s="79">
@@ -9942,13 +9950,13 @@
         <v>1219</v>
       </c>
       <c r="B118" s="30" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="C118" s="76">
         <v>37668</v>
       </c>
       <c r="D118" s="77" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="E118" s="78"/>
       <c r="F118" s="79">
@@ -10028,7 +10036,7 @@
     </row>
     <row r="122" spans="1:35" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B122" s="83" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="C122" s="84">
         <f>COUNTA(B5:B118)</f>
@@ -10041,7 +10049,7 @@
     </row>
     <row r="123" spans="1:35" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B123" s="83" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="C123" s="85">
         <f>SUM(T5:T118)</f>
@@ -10054,7 +10062,7 @@
     </row>
     <row r="124" spans="1:35" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B124" s="83" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="C124" s="86">
         <f>SUM(U5:U118)</f>
@@ -10077,7 +10085,7 @@
     </row>
     <row r="125" spans="1:35" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B125" s="83" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="C125" s="87">
         <f>SUM(C123:C124)</f>
@@ -15352,6 +15360,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <legacyDrawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>